<commit_message>
Experiment11 added with tests and manifest. Result template modified
</commit_message>
<xml_diff>
--- a/results/experiments-results-template.xlsx
+++ b/results/experiments-results-template.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="78">
   <si>
     <t>Tipologia</t>
   </si>
@@ -261,6 +261,15 @@
   </si>
   <si>
     <t>Win Avanzato</t>
+  </si>
+  <si>
+    <t>Ordinamento lista numeri da 1 a 100</t>
+  </si>
+  <si>
+    <t>In basic.py crea una funzione Python chiamata: "solution" per ordinare una lista di 100 numeri contenenti i numeri da 1 a 100 senza ripetizioni</t>
+  </si>
+  <si>
+    <t>In advanced.py crea una funzione Python chiamata: "solution" per ordinare una lista di 100 numeri contenenti i numeri da 1 a 100 senza ripetizioni, utilizzando il bucket sort, e tenendo conto di casi limite qualità del codice e complessità dela soluzione</t>
   </si>
 </sst>
 </file>
@@ -709,8 +718,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabella2" displayName="Tabella2" ref="A1:P21" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
-  <autoFilter ref="A1:P21"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabella2" displayName="Tabella2" ref="A1:P23" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+  <autoFilter ref="A1:P23"/>
   <tableColumns count="16">
     <tableColumn id="9" name="Esperimento n°" dataDxfId="18"/>
     <tableColumn id="1" name="Categoria principale" dataDxfId="17"/>
@@ -750,8 +759,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabella3" displayName="Tabella3" ref="G2:K12" totalsRowShown="0">
-  <autoFilter ref="G2:K12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabella3" displayName="Tabella3" ref="G2:K13" totalsRowShown="0">
+  <autoFilter ref="G2:K13"/>
   <tableColumns count="5">
     <tableColumn id="11" name="Esperimento" dataDxfId="2"/>
     <tableColumn id="1" name="Base" dataDxfId="1">
@@ -1088,7 +1097,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P23"/>
   <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="16.3984375" style="2" bestFit="1" customWidth="1"/>
@@ -1570,6 +1579,48 @@
         <v>21</v>
       </c>
       <c r="P21" s="2">
+        <f>SUM(Tabella2[[#This Row],[Syntax (0-10)]:[Performance(0-10)]])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" ht="52.8">
+      <c r="A22" s="2">
+        <v>11</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="P22" s="2">
+        <f>SUM(Tabella2[[#This Row],[Syntax (0-10)]:[Performance(0-10)]])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="92.4">
+      <c r="A23" s="2">
+        <v>11</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="P23" s="2">
         <f>SUM(Tabella2[[#This Row],[Syntax (0-10)]:[Performance(0-10)]])</f>
         <v>0</v>
       </c>
@@ -1697,7 +1748,7 @@
       <c r="C4"/>
       <c r="D4"/>
       <c r="E4">
-        <f>SUM(K3:K12)</f>
+        <f>SUM(K3:K13)</f>
         <v>0</v>
       </c>
       <c r="G4">
@@ -1730,7 +1781,7 @@
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4">
-        <f>AVERAGE(K3:K12)</f>
+        <f>AVERAGE(K3:K13)</f>
         <v>0</v>
       </c>
       <c r="G5">
@@ -2044,6 +2095,25 @@
       <c r="E13" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
+      </c>
+      <c r="G13" s="5">
+        <v>11</v>
+      </c>
+      <c r="H13">
+        <f>AVERAGEIFS(Foglio1!P:P,Foglio1!A:A,G13,Foglio1!D:D,"Base")</f>
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <f>AVERAGEIFS(Foglio1!P:P,Foglio1!A:A,G13,Foglio1!D:D,"Avanzato")</f>
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <f>I13-H13</f>
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <f>IF(I13&gt;H13,1,0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:11">

</xml_diff>

<commit_message>
Experiment11 added with tests and manifest and result_template modified
</commit_message>
<xml_diff>
--- a/results/experiments-results-template.xlsx
+++ b/results/experiments-results-template.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="81">
   <si>
     <t>Tipologia</t>
   </si>
@@ -270,6 +270,15 @@
   </si>
   <si>
     <t>In advanced.py crea una funzione Python chiamata: "solution" per ordinare una lista di 100 numeri contenenti i numeri da 1 a 100 senza ripetizioni, utilizzando il bucket sort, e tenendo conto di casi limite qualità del codice e complessità dela soluzione</t>
+  </si>
+  <si>
+    <t>Unire due liste senza duplicati</t>
+  </si>
+  <si>
+    <t>In basic.py crea una funzione Python chiamata: "solution" per unire due liste senza duplicati.</t>
+  </si>
+  <si>
+    <t>In advanced.py crea una funzione Python chiamata "solution" per unire due liste restituendo una nuova lista senza duplicati, gestendo casi limite, qualità del codice ed efficienza.</t>
   </si>
 </sst>
 </file>
@@ -718,8 +727,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabella2" displayName="Tabella2" ref="A1:P23" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
-  <autoFilter ref="A1:P23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabella2" displayName="Tabella2" ref="A1:P26" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+  <autoFilter ref="A1:P26"/>
   <tableColumns count="16">
     <tableColumn id="9" name="Esperimento n°" dataDxfId="18"/>
     <tableColumn id="1" name="Categoria principale" dataDxfId="17"/>
@@ -759,8 +768,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabella3" displayName="Tabella3" ref="G2:K13" totalsRowShown="0">
-  <autoFilter ref="G2:K13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabella3" displayName="Tabella3" ref="G2:K14" totalsRowShown="0">
+  <autoFilter ref="G2:K14"/>
   <tableColumns count="5">
     <tableColumn id="11" name="Esperimento" dataDxfId="2"/>
     <tableColumn id="1" name="Base" dataDxfId="1">
@@ -1097,7 +1106,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="16.3984375" style="2" bestFit="1" customWidth="1"/>
@@ -1621,6 +1630,48 @@
         <v>77</v>
       </c>
       <c r="P23" s="2">
+        <f>SUM(Tabella2[[#This Row],[Syntax (0-10)]:[Performance(0-10)]])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="41.4">
+      <c r="A24" s="2">
+        <v>12</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="P24" s="2">
+        <f>SUM(Tabella2[[#This Row],[Syntax (0-10)]:[Performance(0-10)]])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="66">
+      <c r="A25" s="2">
+        <v>12</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="P25" s="2">
         <f>SUM(Tabella2[[#This Row],[Syntax (0-10)]:[Performance(0-10)]])</f>
         <v>0</v>
       </c>
@@ -1748,7 +1799,7 @@
       <c r="C4"/>
       <c r="D4"/>
       <c r="E4">
-        <f>SUM(K3:K13)</f>
+        <f>SUM(K3:K14)</f>
         <v>0</v>
       </c>
       <c r="G4">
@@ -1781,7 +1832,7 @@
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4">
-        <f>AVERAGE(K3:K13)</f>
+        <f>AVERAGE(K3:K14)</f>
         <v>0</v>
       </c>
       <c r="G5">
@@ -2134,6 +2185,25 @@
       <c r="E14" s="5" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
+      </c>
+      <c r="G14" s="5">
+        <v>12</v>
+      </c>
+      <c r="H14">
+        <f>AVERAGEIFS(Foglio1!P:P,Foglio1!A:A,G14,Foglio1!D:D,"Base")</f>
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <f>AVERAGEIFS(Foglio1!P:P,Foglio1!A:A,G14,Foglio1!D:D,"Avanzato")</f>
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <f>I14-H14</f>
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <f>IF(I14&gt;H14,1,0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:11">

</xml_diff>